<commit_message>
feat(saff-study): publish specification and test suite v1.6
</commit_message>
<xml_diff>
--- a/output/xlsx/ExtracaoOffline--GT-.xlsx
+++ b/output/xlsx/ExtracaoOffline--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="72">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -38,7 +38,7 @@
     <t>Reduced (Greedy Heuristic - Transition Coverage)</t>
   </si>
   <si>
-    <t>Size: 9 test case(s)</t>
+    <t>Size: 8 test case(s)</t>
   </si>
   <si>
     <t xml:space="preserve">Creation Date: </t>
@@ -155,6 +155,9 @@
     <t>operador: le (via leitor de codigo de barras) um product number e serial number validos</t>
   </si>
   <si>
+    <t>SYSTEM processes action successfully</t>
+  </si>
+  <si>
     <t>TC6</t>
   </si>
   <si>
@@ -170,61 +173,46 @@
     <t>TC7</t>
   </si>
   <si>
-    <t>Alternative Flow 6: Product number e serial number que nao casam</t>
-  </si>
-  <si>
-    <t>operador: digita um product number e serial number validos mas nao referentes a mesma familia e pressiona Extract (terminal em modo LLT)</t>
-  </si>
-  <si>
-    <t>SYSTEM apresenta mensagem de erro</t>
+    <t xml:space="preserve">Exception Flow 1: Sem conexao e usuario deseja entrar em modo offline </t>
+  </si>
+  <si>
+    <t>SYSTEM exibe mensagem solicitando confirmacao se usuario quer entrar em modo offline</t>
+  </si>
+  <si>
+    <t>operador: confirma que quer entrar em modo offline</t>
+  </si>
+  <si>
+    <t>operador: realiza uma serie de extracoes sequenciais</t>
+  </si>
+  <si>
+    <t>operador: reastabelece conexao</t>
+  </si>
+  <si>
+    <t>SYSTEM envia extracoes locais para o servidor e as apaga da pasta local 'OfflineExtraction'</t>
+  </si>
+  <si>
+    <t>operador: loga no servidor e vai ate a pagina de extracoes</t>
+  </si>
+  <si>
+    <t>SYSTEM exibe lista com extracoes realizadas no modo offline</t>
+  </si>
+  <si>
+    <t>Flow interrupted due to exception / error</t>
   </si>
   <si>
     <t>TC8</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception Flow 1: Sem conexao e usuario deseja entrar em modo offline </t>
-  </si>
-  <si>
-    <t>SYSTEM exibe mensagem solicitando confirmacao se usuario quer entrar em modo offline</t>
-  </si>
-  <si>
-    <t>operador: confirma que quer entrar em modo offline</t>
-  </si>
-  <si>
-    <t>operador: realiza uma serie de extracoes sequenciais</t>
-  </si>
-  <si>
-    <t>operador: reastabelece conexao</t>
-  </si>
-  <si>
-    <t>SYSTEM envia extracoes locais para o servidor e as apaga da pasta local 'OfflineExtraction'</t>
-  </si>
-  <si>
-    <t>operador: loga no servidor e vai ate a pagina de extracoes</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe lista com extracoes realizadas no modo offline</t>
-  </si>
-  <si>
-    <t>Flow interrupted due to exception / error</t>
+    <t xml:space="preserve">Exception Flow 2: Sem conexao e usuario nao deseja entrar em modo offline </t>
+  </si>
+  <si>
+    <t>SYSTEM exibe mensagem solicitando confirmação se usuario quer entrar em modo offline</t>
+  </si>
+  <si>
+    <t>operador: nao deseja entrar em modo offline</t>
   </si>
   <si>
     <t>TC9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exception Flow 2: Sem conexao e usuario nao deseja entrar em modo offline </t>
-  </si>
-  <si>
-    <t>SYSTEM exibe mensagem solicitando confirmação se usuario quer entrar em modo offline</t>
-  </si>
-  <si>
-    <t>operador: nao deseja entrar em modo offline</t>
-  </si>
-  <si>
-    <t>SYSTEM processes action successfully</t>
-  </si>
-  <si>
-    <t>TC10</t>
   </si>
   <si>
     <t>Exception Flow 3: Cai conexao novamente</t>
@@ -331,11 +319,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="114.3671875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="88.19921875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="83.125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>
@@ -808,7 +796,7 @@
         <v>27</v>
       </c>
       <c r="D40" t="s" s="3">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="E40" t="s" s="3">
         <v>27</v>
@@ -830,7 +818,7 @@
         <v>11</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C44" t="s" s="1">
         <v>13</v>
@@ -844,7 +832,7 @@
         <v>15</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E45" t="s" s="1">
         <v>17</v>
@@ -903,13 +891,13 @@
         <v>2.0</v>
       </c>
       <c r="B49" t="s" s="3">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C49" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D49" t="s" s="3">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E49" t="s" s="3">
         <v>27</v>
@@ -951,7 +939,7 @@
         <v>11</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C54" t="s" s="1">
         <v>13</v>
@@ -965,7 +953,7 @@
         <v>15</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E55" t="s" s="1">
         <v>17</v>
@@ -1044,7 +1032,7 @@
         <v>3.0</v>
       </c>
       <c r="B60" t="s" s="3">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="C60" t="s" s="3">
         <v>27</v>
@@ -1064,13 +1052,13 @@
         <v>4.0</v>
       </c>
       <c r="B61" t="s" s="3">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="C61" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D61" t="s" s="3">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E61" t="s" s="3">
         <v>27</v>
@@ -1084,13 +1072,13 @@
         <v>5.0</v>
       </c>
       <c r="B62" t="s" s="3">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="C62" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D62" t="s" s="3">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E62" t="s" s="3">
         <v>27</v>
@@ -1100,118 +1088,118 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="s" s="1">
+      <c r="A63" t="n" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="B63" t="s" s="3">
+        <v>57</v>
+      </c>
+      <c r="C63" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D63" t="s" s="3">
+        <v>58</v>
+      </c>
+      <c r="E63" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F63" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="B64" t="s" s="3">
+        <v>59</v>
+      </c>
+      <c r="C64" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D64" t="s" s="3">
+        <v>60</v>
+      </c>
+      <c r="E64" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F64" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="1">
         <v>33</v>
       </c>
-      <c r="B63" t="s" s="0">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B66" t="s" s="0">
-        <v>55</v>
-      </c>
-      <c r="C66" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E66" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B67" t="s" s="0">
-        <v>56</v>
-      </c>
-      <c r="E67" t="s" s="1">
-        <v>17</v>
+      <c r="B65" t="s" s="0">
+        <v>61</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B68" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="C68" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E68" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B69" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="E69" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B68" t="s" s="0">
+      <c r="B70" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="s" s="2">
+    <row r="71">
+      <c r="A71" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B69" t="s" s="2">
+      <c r="B71" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C69" t="s" s="2">
+      <c r="C71" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D69" t="s" s="2">
+      <c r="D71" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E69" t="s" s="2">
+      <c r="E71" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F69" t="s" s="2">
+      <c r="F71" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B70" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C70" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D70" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E70" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F70" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="n" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="B71" t="s" s="3">
-        <v>29</v>
-      </c>
-      <c r="C71" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D71" t="s" s="3">
-        <v>30</v>
-      </c>
-      <c r="E71" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F71" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n" s="4">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="B72" t="s" s="3">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C72" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D72" t="s" s="3">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="E72" t="s" s="3">
         <v>27</v>
@@ -1222,16 +1210,16 @@
     </row>
     <row r="73">
       <c r="A73" t="n" s="4">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="B73" t="s" s="3">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="C73" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D73" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E73" t="s" s="3">
         <v>27</v>
@@ -1242,16 +1230,16 @@
     </row>
     <row r="74">
       <c r="A74" t="n" s="4">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="B74" t="s" s="3">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="C74" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D74" t="s" s="3">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="E74" t="s" s="3">
         <v>27</v>
@@ -1262,117 +1250,117 @@
     </row>
     <row r="75">
       <c r="A75" t="n" s="4">
-        <v>6.0</v>
+        <v>4.0</v>
       </c>
       <c r="B75" t="s" s="3">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C75" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D75" t="s" s="3">
+        <v>47</v>
+      </c>
+      <c r="E75" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F75" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="B76" t="s" s="0">
         <v>61</v>
       </c>
-      <c r="E75" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F75" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="n" s="4">
-        <v>7.0</v>
-      </c>
-      <c r="B76" t="s" s="3">
-        <v>62</v>
-      </c>
-      <c r="C76" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D76" t="s" s="3">
-        <v>63</v>
-      </c>
-      <c r="E76" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F76" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="s" s="1">
-        <v>33</v>
-      </c>
-      <c r="B77" t="s" s="0">
-        <v>64</v>
+    </row>
+    <row r="79">
+      <c r="A79" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B79" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="C79" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E79" t="s" s="1">
+        <v>14</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="1">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B80" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="C80" t="s" s="1">
-        <v>13</v>
+        <v>67</v>
       </c>
       <c r="E80" t="s" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="1">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B81" t="s" s="0">
-        <v>66</v>
-      </c>
-      <c r="E81" t="s" s="1">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B82" t="s" s="0">
-        <v>19</v>
+      <c r="A82" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B82" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C82" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D82" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E82" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F82" t="s" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B83" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C83" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D83" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E83" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F83" t="s" s="2">
-        <v>25</v>
+      <c r="A83" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B83" t="s" s="3">
+        <v>68</v>
+      </c>
+      <c r="C83" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D83" t="s" s="3">
+        <v>69</v>
+      </c>
+      <c r="E83" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F83" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n" s="4">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="B84" t="s" s="3">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="C84" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D84" t="s" s="3">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="E84" t="s" s="3">
         <v>27</v>
@@ -1383,16 +1371,16 @@
     </row>
     <row r="85">
       <c r="A85" t="n" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B85" t="s" s="3">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="C85" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D85" t="s" s="3">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="E85" t="s" s="3">
         <v>27</v>
@@ -1402,172 +1390,11 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="n" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="B86" t="s" s="3">
-        <v>31</v>
-      </c>
-      <c r="C86" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D86" t="s" s="3">
-        <v>67</v>
-      </c>
-      <c r="E86" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F86" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="n" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="B87" t="s" s="3">
-        <v>68</v>
-      </c>
-      <c r="C87" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D87" t="s" s="3">
-        <v>69</v>
-      </c>
-      <c r="E87" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F87" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="s" s="1">
+      <c r="A86" t="s" s="1">
         <v>33</v>
       </c>
-      <c r="B88" t="s" s="0">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B91" t="s" s="0">
-        <v>70</v>
-      </c>
-      <c r="C91" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E91" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B92" t="s" s="0">
-        <v>71</v>
-      </c>
-      <c r="E92" t="s" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B93" t="s" s="0">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B94" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C94" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D94" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E94" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F94" t="s" s="2">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B95" t="s" s="3">
-        <v>72</v>
-      </c>
-      <c r="C95" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D95" t="s" s="3">
-        <v>73</v>
-      </c>
-      <c r="E95" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F95" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="B96" t="s" s="3">
-        <v>60</v>
-      </c>
-      <c r="C96" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D96" t="s" s="3">
-        <v>74</v>
-      </c>
-      <c r="E96" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F96" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="B97" t="s" s="3">
-        <v>62</v>
-      </c>
-      <c r="C97" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D97" t="s" s="3">
-        <v>75</v>
-      </c>
-      <c r="E97" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F97" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="s" s="1">
-        <v>33</v>
-      </c>
-      <c r="B98" t="s" s="0">
-        <v>64</v>
+      <c r="B86" t="s" s="0">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(saff-study): publish specification and test suite v2.1
</commit_message>
<xml_diff>
--- a/output/xlsx/ExtracaoOffline--GT-.xlsx
+++ b/output/xlsx/ExtracaoOffline--GT-.xlsx
@@ -155,7 +155,7 @@
     <t>TC4</t>
   </si>
   <si>
-    <t xml:space="preserve">Exception Flow 2: Cai conexão e usuario nao quer entrar em modo offline </t>
+    <t xml:space="preserve">Exception Flow 2: Cai conexão e usuario quer entrar em modo offline </t>
   </si>
   <si>
     <t>administrador: não deseja entrar em modo offline</t>
@@ -257,7 +257,7 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="60.25" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="56.78125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="72.93359375" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>

</xml_diff>